<commit_message>
Mise à jour menu via admin (menu Octobre.ods)
</commit_message>
<xml_diff>
--- a/menu_actuel.xlsx
+++ b/menu_actuel.xlsx
@@ -9,38 +9,37 @@
   <sheets>
     <sheet name="Dahl de lentilles corail aux crevettes" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Poke bowl au saumon" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Salade de pois chiches- tomates confites-feta " sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Tarte poireaux saumon" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Croustade aux pommes" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Riz au lait" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Cookies au chocolat" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Crumble pommes fraises" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Crumble pommes poires" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="Pancakes épinards saumon" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Blanquette de Veau" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Pad Thaî au poulet" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="Clafoutis jambon courgettes" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Risotto aux Crevettes" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Quinotto aux Crevettes" sheetId="11" state="visible" r:id="rId11"/>
     <sheet name="Quiche Au Thon" sheetId="12" state="visible" r:id="rId12"/>
     <sheet name="Tortilla quiche au jambon" sheetId="13" state="visible" r:id="rId13"/>
     <sheet name="Crumble salé au poulet" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="Poulet Basquaise" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="Poulet miel soja " sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="Mignon de porc moutarde miel" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="Rougail saucisses" sheetId="16" state="visible" r:id="rId16"/>
     <sheet name="Lasagnes Bolognaise" sheetId="17" state="visible" r:id="rId17"/>
     <sheet name="Risotto aux Champignons" sheetId="18" state="visible" r:id="rId18"/>
     <sheet name="Hachis Parmentier" sheetId="19" state="visible" r:id="rId19"/>
     <sheet name="Chili con Carne" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet name="Curry de Pois Chiches" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet name="Tartiflette" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet name="Quiche Lorraine" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet name="Poulet Coco Curry" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet name="Ratatouille" sheetId="25" state="visible" r:id="rId25"/>
-    <sheet name="Pâtes Carbonara" sheetId="26" state="visible" r:id="rId26"/>
-    <sheet name="Saumon Teriyaki" sheetId="27" state="visible" r:id="rId27"/>
-    <sheet name="Wok Nouilles Crevettes" sheetId="28" state="visible" r:id="rId28"/>
-    <sheet name="Salade César" sheetId="29" state="visible" r:id="rId29"/>
-    <sheet name="Tajine Poulet Citron" sheetId="30" state="visible" r:id="rId30"/>
-    <sheet name="Paella Express" sheetId="31" state="visible" r:id="rId31"/>
-    <sheet name="Gnocchis Pesto Tomates" sheetId="32" state="visible" r:id="rId32"/>
-    <sheet name="Mousse au Chocolat" sheetId="33" state="visible" r:id="rId33"/>
-    <sheet name="Mi-Cuit Chocolat" sheetId="34" state="visible" r:id="rId34"/>
+    <sheet name="Tartiflette" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet name="Quiche Lorraine" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet name="Poulet Coco Curry" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet name="Ratatouille" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet name="Pâtes Carbonara" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet name="Saumon Teriyaki" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet name="Nouilles chinoises aux Crevettes" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet name="Salade César" sheetId="28" state="visible" r:id="rId28"/>
+    <sheet name="Tajine Poulet Citron" sheetId="29" state="visible" r:id="rId29"/>
+    <sheet name="Paella Express" sheetId="30" state="visible" r:id="rId30"/>
+    <sheet name="Gnocchis Pesto Tomates" sheetId="31" state="visible" r:id="rId31"/>
+    <sheet name="Mousse au Chocolat" sheetId="32" state="visible" r:id="rId32"/>
+    <sheet name="Mi-Cuit Chocolat" sheetId="33" state="visible" r:id="rId33"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -765,7 +764,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Riz Arborio</t>
+          <t>Quinoa</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -1316,45 +1315,45 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Filet de poulet</t>
+          <t>Filet de mignon</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>4</v>
+        <v>600</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>pièce(s)</t>
+          <t>g</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Poivron rouge</t>
+          <t>Moutarde</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>pièce(s)</t>
+          <t>càs</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Tomate</t>
+          <t>Miel</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>pièce(s)</t>
+          <t>càs</t>
         </is>
       </c>
     </row>
@@ -1376,26 +1375,26 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Gousse d'ail</t>
+          <t>Crème fraîche</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>2</v>
+        <v>20</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>pièce(s)</t>
+          <t>cl</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Riz</t>
+          <t>Haricots verts</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>240</v>
+        <v>600</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -1414,7 +1413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1450,15 +1449,15 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Filet de Poulet</t>
+          <t>Saucisses</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>600</v>
+        <v>4</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
@@ -1480,11 +1479,11 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Poivrons</t>
+          <t>Oignons</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -1495,30 +1494,45 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Miel</t>
+          <t>Thym</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>60</v>
+        <v>1</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>càs</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Soja</t>
+          <t>Tomates</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>60</v>
+        <v>4</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>ml</t>
+          <t>pièce(s)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Curcuma</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>1</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>càs</t>
         </is>
       </c>
     </row>
@@ -2263,7 +2277,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2274,7 +2288,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Plat végé</t>
+          <t>Plat viande</t>
         </is>
       </c>
       <c r="C1" t="inlineStr"/>
@@ -2299,41 +2313,41 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Pois chiches (conserve)</t>
+          <t>Pomme de terre</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>400</v>
+        <v>1</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>kg</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Lait de coco</t>
+          <t>Reblochon</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>40</v>
+        <v>1</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>cl</t>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Tomates concassées</t>
+          <t>Lardons</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>400</v>
+        <v>200</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -2344,7 +2358,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Pâte de curry</t>
+          <t>Oignon</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -2352,52 +2366,22 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>c.à.s</t>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Riz basmati</t>
+          <t>Crème fraîche</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>250</v>
+        <v>15</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>g</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Oignon</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>2</v>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>pièce(s)</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Coriandre</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>1</v>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>bouquet</t>
+          <t>cl</t>
         </is>
       </c>
     </row>
@@ -2412,7 +2396,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2423,7 +2407,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Plat viande</t>
+          <t>Entrée</t>
         </is>
       </c>
       <c r="C1" t="inlineStr"/>
@@ -2448,7 +2432,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Pomme de terre</t>
+          <t>Pâte brisée</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -2456,67 +2440,82 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>kg</t>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Reblochon</t>
+          <t>Lardons</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1</v>
+        <v>200</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>pièce(s)</t>
+          <t>g</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Lardons</t>
+          <t>Oeuf</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>200</v>
+        <v>3</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Oignon</t>
+          <t>Crème fraîche</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>2</v>
+        <v>20</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>pièce(s)</t>
+          <t>cl</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Crème fraîche</t>
+          <t>Lait</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
           <t>cl</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Emmental</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>150</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>g</t>
         </is>
       </c>
     </row>
@@ -2531,7 +2530,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2542,7 +2541,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Entrée</t>
+          <t>Plat viande</t>
         </is>
       </c>
       <c r="C1" t="inlineStr"/>
@@ -2567,11 +2566,11 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Pâte brisée</t>
+          <t>Filet de poulet</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -2582,73 +2581,58 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Lardons</t>
+          <t>Lait de coco</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>200</v>
+        <v>40</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>cl</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Oeuf</t>
+          <t>Poudre de curry</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>pièce(s)</t>
+          <t>c.à.s</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Crème fraîche</t>
+          <t>Oignon</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>cl</t>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Lait</t>
+          <t>Riz</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>20</v>
+        <v>250</v>
       </c>
       <c r="C7" t="inlineStr">
-        <is>
-          <t>cl</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Emmental</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>150</v>
-      </c>
-      <c r="C8" t="inlineStr">
         <is>
           <t>g</t>
         </is>
@@ -2676,7 +2660,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Plat viande</t>
+          <t>Plat végé</t>
         </is>
       </c>
       <c r="C1" t="inlineStr"/>
@@ -2701,11 +2685,11 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Filet de poulet</t>
+          <t>Courgette</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -2716,22 +2700,22 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Lait de coco</t>
+          <t>Aubergine</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>40</v>
+        <v>2</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>cl</t>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Poudre de curry</t>
+          <t>Poivron</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -2739,18 +2723,18 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>c.à.s</t>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Oignon</t>
+          <t>Tomate</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -2761,15 +2745,15 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Riz</t>
+          <t>Oignon</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>250</v>
+        <v>1</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
@@ -2795,7 +2779,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Plat végé</t>
+          <t>Plat viande</t>
         </is>
       </c>
       <c r="C1" t="inlineStr"/>
@@ -2820,60 +2804,60 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Courgette</t>
+          <t>Spaghetti</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>3</v>
+        <v>400</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>pièce(s)</t>
+          <t>g</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Aubergine</t>
+          <t xml:space="preserve"> Lardons</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>2</v>
+        <v>200</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>pièce(s)</t>
+          <t>g</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Poivron</t>
+          <t>Crème</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>2</v>
+        <v>20</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>pièce(s)</t>
+          <t>cl</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Tomate</t>
+          <t>Pecorino ou Parmesan</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>4</v>
+        <v>100</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>pièce(s)</t>
+          <t>g</t>
         </is>
       </c>
     </row>
@@ -2914,7 +2898,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Plat viande</t>
+          <t>Plat poisson</t>
         </is>
       </c>
       <c r="C1" t="inlineStr"/>
@@ -2939,56 +2923,56 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Spaghetti</t>
+          <t>Pavé de saumon</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>400</v>
+        <v>4</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Lardons</t>
+          <t>Sauce soja</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>200</v>
+        <v>10</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>cl</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Crème</t>
+          <t>Miel</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>cl</t>
+          <t>c.à.s</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Pecorino ou Parmesan</t>
+          <t>Riz basmati</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -2999,7 +2983,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Oignon</t>
+          <t>Brocoli</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -3058,37 +3042,37 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Pavé de saumon</t>
+          <t>Nouilles asiatiques</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>4</v>
+        <v>250</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>pièce(s)</t>
+          <t>g</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Sauce soja</t>
+          <t>Crevettes décortiquées</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>10</v>
+        <v>400</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>cl</t>
+          <t>g</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Miel</t>
+          <t>Carotte</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -3096,22 +3080,22 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>c.à.s</t>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Riz basmati</t>
+          <t>Sauce soja</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>250</v>
+        <v>5</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>cl</t>
         </is>
       </c>
     </row>
@@ -3141,7 +3125,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3152,7 +3136,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Plat poisson</t>
+          <t>Entrée</t>
         </is>
       </c>
       <c r="C1" t="inlineStr"/>
@@ -3177,73 +3161,118 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Nouilles asiatiques</t>
+          <t>Salade Romaine</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>250</v>
+        <v>1</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Crevettes décortiquées</t>
+          <t>Filet de poulet</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>400</v>
+        <v>2</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Carotte</t>
+          <t>Croûtons</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>2</v>
+        <v>100</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>pièce(s)</t>
+          <t>g</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Sauce soja</t>
+          <t>Parmesan</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>5</v>
+        <v>50</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>cl</t>
+          <t>g</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Brocoli</t>
+          <t>Sauce César</t>
         </is>
       </c>
       <c r="B7" t="n">
         <v>1</v>
       </c>
       <c r="C7" t="inlineStr">
+        <is>
+          <t>pot</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Oeuf</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>4</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>pièce(s)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Tomate</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>2</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>pièce(s)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Concombre</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>1</v>
+      </c>
+      <c r="C10" t="inlineStr">
         <is>
           <t>pièce(s)</t>
         </is>
@@ -3271,7 +3300,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Entrée</t>
+          <t>Plat viande</t>
         </is>
       </c>
       <c r="C1" t="inlineStr"/>
@@ -3296,11 +3325,11 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Salade Romaine</t>
+          <t>Cuisse de poulet</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -3311,7 +3340,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Filet de poulet</t>
+          <t>Citron confit</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -3326,7 +3355,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Croûtons</t>
+          <t>Olives vertes</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -3341,22 +3370,22 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Parmesan</t>
+          <t>Oignon</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>50</v>
+        <v>2</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Sauce César</t>
+          <t>Épices Tajine</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -3364,29 +3393,29 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>pot</t>
+          <t>c.à.s</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Oeuf</t>
+          <t>Couscous</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>4</v>
+        <v>500</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>pièce(s)</t>
+          <t>g</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Tomate</t>
+          <t>Courgette</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -3401,7 +3430,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Concombre</t>
+          <t>Poivron</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -3424,7 +3453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3460,41 +3489,41 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Pois chiches</t>
+          <t>Pâte brisée</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>400</v>
+        <v>1</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Tomates confites</t>
+          <t>Poireaux</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>150</v>
+        <v>2</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Feta</t>
+          <t>saumon fumé</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>150</v>
+        <v>200</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -3505,62 +3534,166 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Menthe</t>
+          <t>Oeufs</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>bouquet</t>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Oignons rouges</t>
+          <t>Crème fraîche</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>pièce(s)</t>
+          <t>cl</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Concombre</t>
+          <t>Emmental</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>1</v>
+        <v>100</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>pièce(s)</t>
+          <t>g</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Citron</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>1</v>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>pièce(s)</t>
-        </is>
-      </c>
+      <c r="A9" t="inlineStr"/>
+      <c r="B9" t="inlineStr"/>
+      <c r="C9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr"/>
+      <c r="B10" t="inlineStr"/>
+      <c r="C10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr"/>
+      <c r="B11" t="inlineStr"/>
+      <c r="C11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr"/>
+      <c r="B12" t="inlineStr"/>
+      <c r="C12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr"/>
+      <c r="B13" t="inlineStr"/>
+      <c r="C13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr"/>
+      <c r="B14" t="inlineStr"/>
+      <c r="C14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr"/>
+      <c r="B15" t="inlineStr"/>
+      <c r="C15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr"/>
+      <c r="B16" t="inlineStr"/>
+      <c r="C16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr"/>
+      <c r="B17" t="inlineStr"/>
+      <c r="C17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr"/>
+      <c r="B18" t="inlineStr"/>
+      <c r="C18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr"/>
+      <c r="B19" t="inlineStr"/>
+      <c r="C19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr"/>
+      <c r="B20" t="inlineStr"/>
+      <c r="C20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr"/>
+      <c r="B21" t="inlineStr"/>
+      <c r="C21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr"/>
+      <c r="B22" t="inlineStr"/>
+      <c r="C22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr"/>
+      <c r="B23" t="inlineStr"/>
+      <c r="C23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr"/>
+      <c r="B24" t="inlineStr"/>
+      <c r="C24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr"/>
+      <c r="B25" t="inlineStr"/>
+      <c r="C25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr"/>
+      <c r="B26" t="inlineStr"/>
+      <c r="C26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr"/>
+      <c r="B27" t="inlineStr"/>
+      <c r="C27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr"/>
+      <c r="B28" t="inlineStr"/>
+      <c r="C28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr"/>
+      <c r="B29" t="inlineStr"/>
+      <c r="C29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr"/>
+      <c r="B30" t="inlineStr"/>
+      <c r="C30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr"/>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Pa^te brisée</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3573,7 +3706,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3584,7 +3717,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Plat viande</t>
+          <t>Plat poisson</t>
         </is>
       </c>
       <c r="C1" t="inlineStr"/>
@@ -3609,37 +3742,37 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Cuisse de poulet</t>
+          <t>Riz à paella</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>4</v>
+        <v>300</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>pièce(s)</t>
+          <t>g</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Citron confit</t>
+          <t>Crevettes</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>2</v>
+        <v>200</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>pièce(s)</t>
+          <t>g</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Olives vertes</t>
+          <t>Chorizo</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -3654,22 +3787,22 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Oignon</t>
+          <t>Petit pois</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>2</v>
+        <v>100</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>pièce(s)</t>
+          <t>g</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Épices Tajine</t>
+          <t>Safran ou Spigol</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -3677,50 +3810,35 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>c.à.s</t>
+          <t>dose</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Couscous</t>
+          <t>Cube ou bouillon</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>500</v>
+        <v>1</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Courgette</t>
+          <t>Oignon</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C9" t="inlineStr">
-        <is>
-          <t>pièce(s)</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Poivron</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
-        <v>1</v>
-      </c>
-      <c r="C10" t="inlineStr">
         <is>
           <t>pièce(s)</t>
         </is>
@@ -3737,7 +3855,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3748,7 +3866,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Plat poisson</t>
+          <t>Plat végé</t>
         </is>
       </c>
       <c r="C1" t="inlineStr"/>
@@ -3773,11 +3891,11 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Riz à paella</t>
+          <t>Gnocchis</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>300</v>
+        <v>600</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -3788,11 +3906,11 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Crevettes</t>
+          <t>Pesto vert</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>200</v>
+        <v>150</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -3803,11 +3921,11 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Chorizo</t>
+          <t>Tomates confites</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -3818,60 +3936,15 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Petit pois</t>
+          <t>Parmesan</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
           <t>g</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Safran ou Spigol</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>1</v>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>dose</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Cube ou bouillon</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>1</v>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>pièce(s)</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Oignon</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>1</v>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>pièce(s)</t>
         </is>
       </c>
     </row>
@@ -3886,7 +3959,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3897,7 +3970,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Plat végé</t>
+          <t>Dessert</t>
         </is>
       </c>
       <c r="C1" t="inlineStr"/>
@@ -3922,11 +3995,11 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Gnocchis</t>
+          <t>Chocolat noir</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>600</v>
+        <v>200</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -3937,26 +4010,26 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Pesto vert</t>
+          <t>Oeuf</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>150</v>
+        <v>4</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Tomates confites</t>
+          <t>Sucre</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>250</v>
+        <v>50</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -3967,13 +4040,28 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Parmesan</t>
+          <t>Crème liquide</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="C6" t="inlineStr">
+        <is>
+          <t>cl</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Beurre</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>30</v>
+      </c>
+      <c r="C7" t="inlineStr">
         <is>
           <t>g</t>
         </is>
@@ -4030,125 +4118,6 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>200</v>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>g</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Oeuf</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>4</v>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>pièce(s)</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Sucre</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>50</v>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>g</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Crème liquide</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>20</v>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>cl</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Beurre</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>30</v>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>g</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C7"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Catégorie :</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Dessert</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr"/>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Ingrédient</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Quantité</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Unité</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Chocolat noir</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
         <v>150</v>
       </c>
       <c r="C3" t="inlineStr">
@@ -4574,7 +4543,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4640,15 +4609,15 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Fraises</t>
+          <t>Poires</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>500</v>
+        <v>2</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
@@ -4677,6 +4646,19 @@
         <v>130</v>
       </c>
       <c r="C7" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Poudre amandes50</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr"/>
+      <c r="C8" t="inlineStr">
         <is>
           <t>g</t>
         </is>
@@ -4872,7 +4854,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4908,67 +4890,67 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Viande de veau</t>
+          <t>Poulet</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>800</v>
+        <v>4</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Carotte</t>
+          <t>Nouilles de riz</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>4</v>
+        <v>250</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>pièce(s)</t>
+          <t>g</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Champignon de Paris</t>
+          <t>Sucre Roux</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>250</v>
+        <v>2</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>càs</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Crème fraîche</t>
+          <t>Oignons verts</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>cl</t>
+          <t>botte</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Bouillon de volaille</t>
+          <t>Carotte</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -4976,37 +4958,52 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>cube(s)</t>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Riz</t>
+          <t>Coriandre</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>240</v>
+        <v>1</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>bouquet</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Poireau</t>
+          <t>Sauce teriyaki</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>2</v>
+        <v>30</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>pièce(s)</t>
+          <t>g</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Cacahuètes</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>30</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>g</t>
         </is>
       </c>
     </row>

</xml_diff>